<commit_message>
Un riassunto per ciascuno dei 147 giochi
Nuova colonna Descrizione nel foglio Giochi, con due righe per titolo scritte
rielaborando schede di BoardGameGeek, La Tana dei Goblin e siti degli editori:
raccontano che cosa si fa davvero durante una partita.

- Ogni riga dell'elenco ora si apre e mostra il riassunto sopra le espansioni;
  prima erano apribili solo i giochi che avevano espansioni.
- La ricerca testuale considera anche le descrizioni.
- Il modulo di gestione ha il campo Descrizione, salvato nel file Excel.
- I testi stanno in tools/descrizioni.py, separati dai dati numerici.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dati/giochi.xlsx
+++ b/dati/giochi.xlsx
@@ -139,16 +139,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TabellaGiochi" displayName="TabellaGiochi" ref="A1:G148" headerRowCount="1">
-  <autoFilter ref="A1:G148"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TabellaGiochi" displayName="TabellaGiochi" ref="A1:H148" headerRowCount="1">
+  <autoFilter ref="A1:H148"/>
+  <tableColumns count="8">
     <tableColumn id="1" name="Nome"/>
     <tableColumn id="2" name="Giocatori min"/>
     <tableColumn id="3" name="Giocatori max"/>
     <tableColumn id="4" name="Durata min"/>
     <tableColumn id="5" name="Durata max"/>
     <tableColumn id="6" name="Tag"/>
-    <tableColumn id="7" name="Note"/>
+    <tableColumn id="7" name="Descrizione"/>
+    <tableColumn id="8" name="Note"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -466,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G148"/>
+  <dimension ref="A1:H148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -475,7 +476,8 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="90" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,6 +513,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Descrizione</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
@@ -538,6 +545,11 @@
           <t>Cooperativo, Deduzione, Investigazione, Party game</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Quindici minuti per risolvere un caso: si fanno domande a chi conosce la verità, che può rispondere solo sì o no, fino a ricostruire i tre segreti nascosti.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -562,6 +574,11 @@
           <t>Gioco di carte, Memoria, Filler, Push your luck</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Si raccolgono carte dei sette peccati ricordando quelle già passate: eccedere in un vizio condanna all'abisso, restare troppo virtuosi non paga. Conta la misura.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -586,6 +603,11 @@
           <t>Gioco di carte, Astratto, Filler</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Ogni carta giocata cambia la regola che stabilisce chi sta vincendo: al termine del proprio turno bisogna trovarsi in testa secondo la regola del momento, o si è fuori.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -610,6 +632,11 @@
           <t>Eurogame, Draft, Gioco di carte, Storico, Civilizzazione</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Tre ere di civiltà giocate a mano passante: si sceglie una carta e si cede il resto al vicino, costruendo intanto risorse, esercito, scienza e la propria meraviglia.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -634,6 +661,11 @@
           <t>Eurogame, Per due, Draft, Gioco di carte, Storico</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>7 Wonders rifatto per due: le carte sono disposte a piramide e si possono prendere solo quelle libere. Si vince ai punti, ma anche con l'esercito o con la scienza.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -658,6 +690,11 @@
           <t>Party game, Ruoli nascosti, Bluff, Deduzione</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>I fedeli di Artù devono portare a termine le missioni, gli scagnozzi di Mordred sabotarle. Merlino sa chi sono i cattivi, ma se si fa scoprire fa perdere la sua squadra.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -682,6 +719,11 @@
           <t>Party game, Umoristico, Per adulti</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Domande scomode sul gruppo: si vota chi fra i presenti corrisponde meglio alla descrizione. Da giocare solo con chi sa prenderla bene.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -706,6 +748,11 @@
           <t>Push your luck, Filler, Family game</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Si pescano patatine colorate dal sacchetto e si scommette su quali obiettivi si riuscirà a completare, scartando per tempo quelli ormai diventati impossibili.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -730,6 +777,11 @@
           <t>Parole, Rapidità, Family game, Solitario</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Ognuno costruisce il proprio cruciverba con le tessere lettera, senza turni e senza aspettare: quando qualcuno finisce i pezzi, tutti ne pescano un altro.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -754,6 +806,11 @@
           <t>Ruoli nascosti, Gioco di carte, Party game, Western, Bluff</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Far West a ruoli nascosti: lo sceriffo è allo scoperto, fuorilegge, vice e rinnegato no. Si spara a distanza di carte cercando di capire chi vuole davvero la tua pelle.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -778,6 +835,11 @@
           <t>Party game, Quiz, Push your luck, A squadre, Family game</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Quiz con risposte numeriche da zero a dieci: si stima il valore nascosto e si decide se tenere la carta o passare, cercando di avvicinarsi a ventuno senza sballare.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -802,6 +864,11 @@
           <t>Eurogame, Gestione risorse, Solitario, Gioco pesante</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Si colonizza una terra selvaggia costruendo case, allevando animali e innescando catene di azioni sempre più efficienti. Ci si sposta solo dove sono già passati gli altri.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -826,6 +893,11 @@
           <t>Party game, Destrezza, Tempo reale, Family game, Umoristico</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Si scambiano carte alla ricerca di tris e, quando salta fuori la carta duello, si afferra il burrito di gommapiuma e lo si tira addosso all'avversario. Caos garantito.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -850,6 +922,11 @@
           <t>Gioco di carte, Push your luck, Filler, Party game</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Si gioca una carta per volta su una fila comune: superare ventuno fa saltare il banco e chi ha causato il disastro resta a mani vuote mentre gli altri incassano.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -874,6 +951,11 @@
           <t>Family game, Party game, Scommesse, Dadi, Push your luck</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Cammelli che si accavallano in groppa l'uno all'altro e scommesse da piazzare al momento giusto: si punta sulla tappa, sul vincitore finale e persino su chi arriverà ultimo.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -898,6 +980,11 @@
           <t>Party game, A squadre, Tempo reale, Deduzione</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Due sottomarini, due squadre, tutto in tempo reale: capitano, ufficiale, radarista e ingegnere devono coordinarsi a voce, nel caos, per localizzare e affondare l'avversario.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -922,6 +1009,11 @@
           <t>Eurogame, Family game, Piazzamento tessere, Classico</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Si pesca una tessera e la si incastra nel paesaggio, poi si decide se piazzarci sopra un omino per rivendicare una strada, una città o un monastero. I confini contano più del resto.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -946,6 +1038,11 @@
           <t>Family game, Corsa, Gestione mano, Pirati</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Evasione dal forte: si scartano carte per far avanzare i pirati verso la barca, ma per recuperarne bisogna tornare indietro. O si esce tutti, o non è uscito nessuno.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -970,6 +1067,11 @@
           <t>Party game, Bluff, Negoziazione, Umoristico</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Tutti puntano una pistola di gommapiuma contro qualcuno e devono decidere in un istante se restare o tirarsi indietro. Chi resta in piedi si spartisce il bottino.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -994,6 +1096,11 @@
           <t>Deckbuilder, Gioco di carte, Family game, Torneo</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Un torneo a eliminazione: ogni round si aggiungono carte al proprio mazzo e lo si fa scontrare in automatico con quello dell'avversario di turno. Tutti giocano insieme e alla fine restano due in finale.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1018,6 +1125,11 @@
           <t>Gioco di carte, Prese, Per due, Filler, Fantasy</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Prese in due divise in due tempi: nella prima metà si vincono le carte che formeranno il proprio esercito, nella seconda si combatte proprio con quello che si è raccolto.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1042,6 +1154,11 @@
           <t>Gioco di carte, Set collection, Family game, Filler</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Si aggiungono carte alle file oppure se ne prende una intera: alla fine solo tre colori danno punti e gli altri li tolgono. Decidere quando fermarsi è tutto il gioco.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1066,6 +1183,11 @@
           <t>Family game, Programmazione, Western, Party game</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Si programmano in anticipo le mosse dei banditi su un treno tridimensionale, poi si esegue tutto nell'ordine stabilito — e quasi mai come lo si era immaginato.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1090,6 +1212,11 @@
           <t>Party game, Family game, Rapidità, Bambini</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Una serie di prove lampo — memoria, percorsi, tatto, logica, calcolo — in cui conta solo arrivare per primi con la risposta giusta, prima ancora di aver capito la domanda.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1114,6 +1241,11 @@
           <t>Controllo territorio, Asimmetrico, Negoziazione, Eurogame, Gioco pesante</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Medio Oriente del X secolo: cinque fazioni molto diverse — sultano, califfo, nomadi, signore della guerra, cospiratore — si contendono il territorio fra alleanze temporanee, favori comprati e tradimenti.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1138,6 +1270,11 @@
           <t>Deduzione, Investigazione, Family game, Logica</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Ognuno conosce un solo indizio sulla posizione della creatura. A turno si fanno domande e si escludono caselle, finché qualcuno incrocia abbastanza informazioni da trovarla.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1162,6 +1299,11 @@
           <t>Dadi, Classico, Push your luck, Family game, Solitario</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Cinque dadi con i semi delle carte: si tira fino a tre volte cercando la combinazione migliore — scala, full, poker — e si segna il punteggio sul foglio.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1186,6 +1328,11 @@
           <t>Escape room, Cooperativo, Gioco di carte, Enigmi, Solitario</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Variante competitiva della serie: due ciurme giocano lo stesso mazzo fianco a fianco e vince chi risolve gli enigmi piratereschi commettendo meno errori.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1210,6 +1357,11 @@
           <t>Escape room, Cooperativo, Gioco di carte, Enigmi, Solitario</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Escape room in un mazzo di carte, da giocare in gruppo senza preparazione: enigmi da risolvere insieme per evadere dal carcere più duro d'America.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1234,6 +1386,11 @@
           <t>Escape room, Cooperativo, Gioco di carte, Enigmi, Solitario</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Escape room contenuta in un mazzo di carte: si legge, si discute e si decide insieme, e ogni errore costa tempo. Qui si indaga su un complotto fra le strade di Londra.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1258,6 +1415,11 @@
           <t>Escape room, Cooperativo, Gioco di carte, Enigmi, Solitario</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Escape room in un mazzo di carte: si attraversa la giungla sulle tracce della città d'oro, risolvendo enigmi in gruppo e pagando ogni errore in tempo perso.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1282,6 +1444,11 @@
           <t>Escape room, Cooperativo, Gioco di carte, Enigmi, Solitario</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Il primo della serie: chiusi in un laboratorio, si risolvono insieme gli enigmi di un test che si rivela più insidioso del previsto. Bastano il mazzo e un tavolo.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1306,6 +1473,11 @@
           <t>Party game, A squadre, Deduzione, Parole</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>La propria squadra deve capire il codice dai tuoi indizi, l'altra ascolta e prova a intercettarlo. Più indizi dai nel corso della partita, più rischi di farti decifrare.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1330,6 +1502,11 @@
           <t>Party game, Family game, Creatività, Gioco di carte</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Il narratore descrive con una frase una delle sue illustrazioni oniriche; gli altri giocano una carta che possa ingannare e poi tutti votano. Si guadagna solo se qualcuno indovina, ma non se indovinano tutti.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1354,6 +1531,11 @@
           <t>Party game, Rapidità, Osservazione, Family game, Bambini, Filler</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Fra due carte qualsiasi c'è sempre un solo simbolo in comune: vince chi lo vede e lo nomina per primo. Cinque modi di giocare, cinque minuti a partita.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1378,6 +1560,11 @@
           <t>Astratto, Classico, Family game</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Le tessere si accostano per numeri uguali, allungando una catena in entrambe le direzioni finché qualcuno non riesce più a muovere o esaurisce la mano.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1402,6 +1589,11 @@
           <t>Cooperativo, Tempo reale, Party game, Filler, Umoristico</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Cinque minuti di panico cooperativo in tempo reale: bisogna portare l'eroe al bagno prima che scada la clessidra, superando i mostri che si mettono in mezzo.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1426,6 +1618,11 @@
           <t>Gioco di carte, Party game, Memoria, Umoristico, Family game</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Memory a tema Fantozzi: si accoppiano scene e battute dei primi due film, con l'effetto comico che fa buona parte del lavoro al posto delle regole.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1450,6 +1647,11 @@
           <t>Gioco di carte, Eurogame, Draft, Filler</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Si gioca una carta per notte e alla fine si leggono i propri obiettivi al contrario: conta ciò che si è messo prima, quindi bisogna ragionare sulla partita a ritroso.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1474,6 +1676,11 @@
           <t>Destrezza, Family game, Western, A squadre</t>
         </is>
       </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Far West a schicchere: si spara ai barili e ai banditi con un colpo di dito, si cavalca, si rapina la banca. Tutto si risolve con la mira, non con i dadi.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1498,6 +1705,11 @@
           <t>Deckbuilder, Gioco di carte, Eurogame, Family game</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Si mette insieme una banda di bambini giocando carte, ma quelle che non si usano possono essere prese dagli altri: il mazzo va sfruttato tutto, e va sfruttato in fretta.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1522,6 +1734,11 @@
           <t>Astratto, Per due, Classico, Family game</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Il classico a gravità: si lasciano cadere i gettoni nelle colonne cercando di allinearne quattro in orizzontale, verticale o diagonale prima dell'avversario.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1546,6 +1763,11 @@
           <t>Family game, Corsa, Interazione cattiva, Horror</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Si guida un gruppetto di personaggi fuori da un sotterraneo mentre un mostro li insegue; massi da spingere, pozze scivolose e teletrasporti complicano ogni fuga.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1570,6 +1792,11 @@
           <t>Family game, Classico, Tira e muovi, Economico</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Un mese di calendario da attraversare fra bollette, affari e imprevisti; a fine mese arriva lo stipendio e si saldano i debiti. Vince chi ha messo da parte di più.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1594,6 +1821,11 @@
           <t>Gioco di carte, Narrativo, Umoristico, Party game</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Si racconta la vita sempre più sfortunata della propria famiglia gotica: si accumulano disgrazie sui propri personaggi e poi li si manda incontro a una fine adeguatamente tragica.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1618,6 +1850,11 @@
           <t>Gioco di carte, Party game, Umoristico, Filler</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Rivoluzione francese in chiave comica: si riordina la fila dei nobili in attesa del patibolo per accaparrarsi, al proprio turno, le teste che valgono di più.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1642,6 +1879,11 @@
           <t>Gioco di carte, Party game, Umoristico, Family game</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Dinosauri che cercano di sopravvivere a meteore e disgrazie assortite: si schivano i disastri con le carte in mano e si spera che tocchi a qualcun altro.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1666,6 +1908,11 @@
           <t>Astratto, Per due, Classico</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Scacchi senza scacchiera: si posano tessere esagonali con insetti, ognuno con un movimento proprio, per accerchiare completamente l'ape regina avversaria.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1690,6 +1937,11 @@
           <t>Party game, Rapidità, Gioco di carte, Family game</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Si conta da uno a sette e ritorno scoprendo carte, ma i personaggi raffigurati cambiano le regole al volo: chi sbaglia il conto si prende tutto il mazzetto.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1714,6 +1966,11 @@
           <t>Party game, Destrezza, Family game, Bambini</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Si vincono uova con piccole prove di destrezza e poi bisogna tenerle addosso — sotto il mento, fra le ginocchia, nell'incavo del braccio — mentre la partita continua.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1738,6 +1995,11 @@
           <t>Gioco di carte, Party game, Family game, Grandi gruppi</t>
         </is>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Gerarchia spietata: si scartano gruppi di carte uguali per liberarsi la mano e a fine round si cambia posto al tavolo. Il primo comanda, l'ultimo mescola e serve da bere.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1762,6 +2024,11 @@
           <t>Party game, Umoristico, Per adulti, A squadre, Grandi gruppi</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Un tram fuori controllo e due binari: due squadre argomentano per convincere il macchinista a schiacciare gli altri. Il dilemma del carrello, in versione irriverente.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1786,6 +2053,11 @@
           <t>Party game, Creatività, Deduzione</t>
         </is>
       </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Si compone un'immagine sovrapponendo e muovendo carte trasparenti per far indovinare un film, un personaggio, un modo di dire. Niente parole, solo forme.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1810,6 +2082,11 @@
           <t>Party game, Bluff, Memoria, Gioco di carte</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>A tavola con un veleno in mano: si passano e si scambiano carte per avvelenare il proprio bersaglio, bere più vino degli altri e soprattutto arrivare vivi al brindisi finale.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1834,6 +2111,11 @@
           <t>Gioco di carte, Bluff, Filler, Family game</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Tre carte per turno: una davanti a sé, una davanti a un avversario e una sul tavolo della regina. Bisogna far salire le famiglie giuste e affondare quelle degli altri.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1858,6 +2140,11 @@
           <t>Party game, Cooperativo, Parole, Family game, Grandi gruppi</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Una parola da indovinare, tutti scrivono un indizio di una parola sola — e gli indizi identici si cancellano a vicenda. Cooperativo: si vince o si perde insieme.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1882,6 +2169,11 @@
           <t>Eurogame, Per due, Controllo territorio, Gioco di carte</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Duello sulle isole del Pacifico: si giocano carte per costruire ponti e, quando si conquista la maggioranza dei collegamenti di un'isola, quelli dell'altro vengono spazzati via.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1906,6 +2198,11 @@
           <t>Astratto, Per due, Filler</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Astratto per due senza alcuna casualità: il colore della casella su cui arrivi decide con quale pezzo l'avversario dovrà muovere. Vince chi raggiunge per primo il lato opposto.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1930,6 +2227,11 @@
           <t>Family game, Scommesse, Bluff, Eurogame</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Si muovono nobili condivisi verso il trono scommettendo di nascosto su chi arriverà in alto: conviene spingere anche i candidati degli altri per non farsi scoprire.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1954,6 +2256,11 @@
           <t>Family game, Piazzamento tessere, Draft, Eurogame</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Si scelgono tessere a due caselle in ordine di forza e le si incastra nel proprio regno cinque per cinque, accostando terreni uguali e concentrandoci sopra le corone.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1978,6 +2285,11 @@
           <t>Destrezza, Filler, Party game, Family game</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Sassi magnetici da posare uno alla volta dentro un cordoncino: se si attirano fra loro, chi li ha fatti scattare se li riprende in mano. Vince chi li piazza tutti.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2002,6 +2314,11 @@
           <t>Gioco di carte, Family game, Filler, Pirati</t>
         </is>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Galeoni carichi d'oro e pirati di quattro colori: si accumulano forze su una nave e si incassa il bottino quando, al proprio turno, si ha la maggioranza.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2026,6 +2343,11 @@
           <t>Party game, Horror, Gioco di carte, Interazione cattiva, Umoristico</t>
         </is>
       </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Chiusi in una villa maledetta, si passa di stanza in stanza per raccogliere monete e, all'occorrenza, per togliere di mezzo qualcun altro. Solo carte, molto rumore.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2050,6 +2372,11 @@
           <t>Party game, Parole, Cooperativo, Comunicazione limitata</t>
         </is>
       </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Nella giungla si indica un percorso ai compagni usando una parola per volta: chi ascolta deve collegare gli indizi e ricostruire la strada giusta verso il tesoro.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2074,6 +2401,11 @@
           <t>Dadi, Party game, Family game, Push your luck, Scommesse</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Si piazzano i propri dadi nei casinò e chi ha la maggioranza in uno ne incassa il premio. Il difficile è capire dove insistere e dove lasciar perdere, perché due pari merito si annullano.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2098,6 +2430,11 @@
           <t>American, Horror, Movimento nascosto, Uno contro tutti, Deduzione</t>
         </is>
       </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Omaggio agli slasher anni Ottanta: un giocatore muove l'assassino in segreto su una mappa, gli altri sono i ragazzi che cercano di sopravvivere e di intuirne il percorso. Si gioca in quattro capitoli concatenati.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2122,6 +2459,11 @@
           <t>Party game, Ruoli nascosti, Bluff, Deduzione</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Due clan di vampiri mescolati nella stessa stanza: si attacca, si deduce e si sospetta, finché uno dei due non riesce a identificare e catturare il capo avversario.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2146,6 +2488,11 @@
           <t>Party game, Ruoli nascosti, Bluff, Deduzione, Grandi gruppi</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Il classico da gruppo numeroso: di notte i lupi scelgono una vittima, di giorno il villaggio discute e vota chi eliminare. Serve qualcuno che faccia da narratore.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2170,6 +2517,11 @@
           <t>Party game, Ruoli nascosti, Bluff, Deduzione</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Lupus in tabula concentrato per gruppi piccoli: di notte il lupo mannaro colpisce, di giorno il villaggio lincia un sospetto, e i ruoli speciali cambiano a ogni partita.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2194,6 +2546,11 @@
           <t>Party game, Bluff, Deduzione, Gioco di carte, Filler</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Cinque animali in ordine di forza e tutti giocano una carta coperta. Quando il proprio animale viene chiamato bisogna svelarsi e provare a mangiare chi sta più in basso.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2218,6 +2575,11 @@
           <t>Asimmetrico, Gioco di carte, American, Family game</t>
         </is>
       </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Ogni cattivo ha obiettivo e mazzo suoi: si persegue il proprio piano mentre gli altri ti mettono i bastoni fra le ruote giocando carte destino contro di te.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2242,6 +2604,11 @@
           <t>Party game, Bluff, Ruoli nascosti, Memoria</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Tutti conoscono il proprio ruolo, poi le carte vengono scambiate sotto il tavolo e nessuno è più sicuro di niente. Si dichiara un personaggio e si aspetta chi smentisce.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2266,6 +2633,11 @@
           <t>Gioco di carte, Bluff, Filler, Family game</t>
         </is>
       </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Si dichiara quello che si sta giocando, ma nessuno controlla finché qualcuno non chiama il bluff. Poche carte, venti minuti e parecchie bugie.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2290,6 +2662,11 @@
           <t>Party game, Cooperativo, Quiz, Family game, Solitario</t>
         </is>
       </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Stessa formula di Match Up! con un mazzo dedicato alla cucina: indizi da leggere ad alta voce e parole da abbinare, in cooperativa e a difficoltà regolabile.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2314,6 +2691,11 @@
           <t>Party game, Cooperativo, Quiz, Family game, Solitario</t>
         </is>
       </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Si dispongono le carte parola sul tavolo e si associano agli indizi letti a voce alta, tutti insieme, scegliendo quanto rendersi la vita difficile.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2338,6 +2720,11 @@
           <t>Wargame, Storico, Per due, Dadi, Gioco di carte</t>
         </is>
       </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Seconda guerra mondiale in miniatura: le carte comando dicono su quale settore del fronte si può agire e i dadi risolvono gli scontri. Ogni scenario ricostruisce una battaglia realmente avvenuta.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2362,6 +2749,11 @@
           <t>Cooperativo, Investigazione, Osservazione, Family game, Solitario</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Una mappa enorme piena di scenette: le carte pongono domande su un delitto e la risposta va cercata fra le figure, seguendo i personaggi da un angolo all'altro della città.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2386,6 +2778,11 @@
           <t>Family game, Bambini, Dadi, Labirinto</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Labirinto di mattoncini che cambia forma: si tira il dado per portare i propri eroi al tempio, spostando i muri e scatenando il minotauro sui personaggi degli altri.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2410,6 +2807,11 @@
           <t>Gioco di carte, Umoristico, Party game, Interazione cattiva</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Carte assurde giocabili in qualsiasi momento, anche nel turno degli altri: si accumulano oggetti e si sabota chi sta per vincere, spesso all'ultimo secondo utile.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2434,6 +2836,11 @@
           <t>Gioco di carte, Umoristico, Interazione cattiva, Party game, Horror</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Si scende nel dungeon per salire di livello, ma soprattutto per sabotare gli altri sul più bello. Parodia, carte cattive e nessuna pietà per chi sta per vincere.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2458,6 +2865,11 @@
           <t>Cooperativo, Deduzione, Comunicazione limitata, Horror</t>
         </is>
       </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Un fantasma comunica solo con grandi carte illustrate oniriche; i medium devono interpretarle per ricostruire assassino, arma e luogo prima che scadano le notti.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2482,6 +2894,11 @@
           <t>Gioco di carte, Prese, Eurogame, A squadre</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Prima di giocare le carte si decide insieme, eliminando un'opzione per volta, quali saranno le regole della mano: atout, valore delle prese, chi comincia, quanto si scarta.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2506,6 +2923,11 @@
           <t>Party game, Parole, A squadre, Deduzione</t>
         </is>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Due squadre, una griglia di parole e un capitano che può dire una sola parola e un numero per far indovinare più agenti possibile — evitando a ogni costo l'assassino.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2530,6 +2952,11 @@
           <t>Party game, A squadre, Deduzione, Osservazione</t>
         </is>
       </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Come Nome in codice, ma la griglia è fatta di illustrazioni piene di dettagli: l'indizio deve agganciare quello che si vede, non quello che si legge.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2554,6 +2981,11 @@
           <t>Classico, Family game, Dadi, Tira e muovi</t>
         </is>
       </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Il gioco della tradizione: si tirano i dadi per portare le proprie quattro pedine dal via al traguardo, rispedendo a casa chi si trova sulla casella d'arrivo.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2578,6 +3010,11 @@
           <t>Uno contro tutti, Gioco di carte, Fantascienza, Bluff</t>
         </is>
       </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Un giocatore è la Creatura che dà la caccia, gli altri sono i naufraghi che si nascondono giocando in segreto i luoghi dell'isola, sperando di non incrociarla.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2602,6 +3039,11 @@
           <t>Gioco di carte, Per due, Filler, Family game</t>
         </is>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Tiro alla fune in due: a ogni mano si divide il mazzetto e se ne passa metà all'avversario, poi si giocano le carte forza per aggiudicarsi i barili in palio.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2626,6 +3068,11 @@
           <t>Astratto, Per due, Filler</t>
         </is>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Duello astratto fra zeri e uni: si posano carte nelle righe di codice e si usano i comandi per ribaltare la situazione prima che il programma venga eseguito.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2650,6 +3097,11 @@
           <t>Gioco di carte, Bluff, Programmazione, Filler, Medievale</t>
         </is>
       </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Si dispone una fila di personaggi coperti: ognuno può essere rivelato per usarne il potere oppure lasciato nascosto per incassare influenza, indovinando le mosse degli altri.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2674,6 +3126,11 @@
           <t>Astratto, Per due, Classico</t>
         </is>
       </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Un minuto per impararlo, una vita per padroneggiarlo: si racchiudono le pedine avversarie fra due proprie per capovolgerle. Vince chi alla fine ne ha di più del suo colore.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2698,6 +3155,11 @@
           <t>Eurogame, Controllo territorio, Filler</t>
         </is>
       </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Un gioco di conquista ridotto all'osso: poche azioni a testa, una manciata di minuti e la mappa è già decisa fra truppe piazzate e carte merce raccolte.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2722,6 +3184,11 @@
           <t>Parole, Classico, Family game, Rapidità</t>
         </is>
       </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Si agita la griglia di dadi con le lettere e in un minuto si scrivono più parole possibile collegando lettere adiacenti. Le parole trovate anche da altri non contano.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2746,6 +3213,11 @@
           <t>Eurogame, Set collection, Piazzamento tessere, Arte</t>
         </is>
       </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Si mescolano colori primari come su una tavolozza per riprodurre la gamma di quadri famosi e incassare le commissioni. Elegante, e si impara qualcosa di storia dell'arte.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2770,6 +3242,11 @@
           <t>Dadi, Bluff, Party game, Classico</t>
         </is>
       </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Si dichiara quanti dadi di un certo valore ci sono sotto tutti i bicchieri del tavolo, rilanciando oppure smascherando chi ha esagerato. Il bluff dei pirati.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2794,6 +3271,11 @@
           <t>Party game, Family game, Osservazione, Bambini</t>
         </is>
       </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Caccia al dettaglio su tabelloni affollati di oggetti disegnati alla rinfusa: le carte chiedono di trovarne uno e vince chi lo individua per primo. Alcune missioni si giocano a tempo, altre a colpo d'occhio.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2818,6 +3300,11 @@
           <t>Eurogame, Family game, Puzzle, Set collection</t>
         </is>
       </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Si sfilano le biglie da un distributore verticale: ogni presa fa franare le altre e può innescare reazioni a catena. Con gli ingredienti raccolti si completano le pozioni richieste.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2842,6 +3329,11 @@
           <t>Party game, Deduzione, Bluff, A squadre, Comunicazione limitata</t>
         </is>
       </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Uno speaker descrive due carte con una frase in codice: la propria squadra deve riconoscerle, l'altra ascolta e prova a intercettare il messaggio prima di loro.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2866,6 +3358,11 @@
           <t>Party game, Fantasy, Filler, Umoristico</t>
         </is>
       </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>I maghi si contendono il tesoro lanciandosi incantesimi decisi con le dita, alla morra cinese: si conta fino a tre e si scopre chi ha colpito chi.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2890,6 +3387,11 @@
           <t>Astratto, Puzzle, Logica, Solitario, Family game</t>
         </is>
       </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Un rompicapo collettivo: tutti guardano la stessa griglia e cercano in quante mosse portare un robot all'obiettivo, sapendo che i robot scivolano finché non urtano qualcosa.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2914,6 +3416,11 @@
           <t>Cooperativo, Ruoli nascosti, Fantascienza, Programmazione, Solitario</t>
         </is>
       </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Rinchiusi in un complesso di stanze mortali, si programmano le mosse per trovare l'uscita — sapendo che qualcuno del gruppo potrebbe lavorare per i carcerieri.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2938,6 +3445,11 @@
           <t>Controllo territorio, Asimmetrico, Wargame, Gioco pesante, Fantasy</t>
         </is>
       </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Sotto l'aspetto di una favola animale c'è un conflitto profondamente asimmetrico: gatti industriali, uccelli in guerra, ribelli della foresta e un vagabondo giocano con regole e obiettivi completamente diversi.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2962,6 +3474,11 @@
           <t>Per due, Filler, Astratto</t>
         </is>
       </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Astratto secco per due: nove regni disposti in griglia e sette carte a testa da giocare per rivendicarli. Quando la griglia è piena vince chi ne controlla di più.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2986,6 +3503,11 @@
           <t>Family game, Corsa, Fantasy, Interazione cattiva</t>
         </is>
       </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Corse demenziali su circuiti con vulcani e ponti sospesi: ogni carta dà insieme un movimento e un effetto — missili, mine, riparazioni — da usare al momento giusto.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3010,6 +3532,11 @@
           <t>Eurogame, Family game, Dadi, Puzzle, Draft</t>
         </is>
       </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Si costruisce una vetrata incastonando dadi colorati in una griglia che impone vincoli di colore e di valore. Un puzzle silenzioso, giocato con quello che gli altri hanno lasciato.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3034,6 +3561,11 @@
           <t>Astratto, Eurogame, Gestione mano, Medievale</t>
         </is>
       </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Sopra un abisso, monaci camminano su passerelle mobili: si giocano carte per ruotare i ponti e raggiungere i propri quattro libri prima degli avversari.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3058,6 +3590,11 @@
           <t>Astratto, Per due, Classico</t>
         </is>
       </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Il gioco di strategia per eccellenza: sedici pezzi per parte, nessun elemento casuale e un solo obiettivo, mettere sotto scacco matto il re avversario.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3082,6 +3619,11 @@
           <t>Eurogame, Controllo territorio, Gestione risorse, Piazzamento lavoratori, Solitario, Gioco pesante</t>
         </is>
       </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Europa alternativa degli anni Venti, fra contadini e mech a vapore: si alternano azioni su una plancia personale per produrre, espandersi e combattere, piazzando le proprie stelle prima degli altri.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3106,6 +3648,11 @@
           <t>Gioco di carte, Family game, Push your luck, Filler, Classico</t>
         </is>
       </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Quattro file sul tavolo e carte numerate da piazzare: chi appoggia la sesta carta di una fila si porta via tutte le precedenti con i loro punti di penalità.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3130,6 +3677,11 @@
           <t>Party game, Umoristico, Per adulti, Gioco di carte</t>
         </is>
       </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Si ordinano le disgrazie della vita quotidiana secondo quanto sono terribili, discutendo animatamente su che cosa sia davvero peggio. Per adulti, senza filtri.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3154,6 +3706,11 @@
           <t>Cooperativo, Deduzione, Gioco di carte, Filler</t>
         </is>
       </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Un giocatore dà indizi mostrando altre carte e dicendo soltanto se somigliano o no al personaggio segreto; insieme si scartano le carte fino a isolare quella giusta.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3178,6 +3735,11 @@
           <t>Cooperativo, Deduzione, Gioco di carte, Filler</t>
         </is>
       </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Stessa meccanica di Similo su un nuovo mazzo: indizi per somiglianza e per differenza, dodici carte sul tavolo e un numero limitato di tentativi per arrivare a quella giusta.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3202,6 +3764,11 @@
           <t>Party game, Bluff, Filler, Gioco di carte</t>
         </is>
       </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Si punta fiore o teschio a faccia in giù, poi si scommette su quante carte si riesce a scoprire senza trovare un teschio. Nessun tabellone: solo bluff e facce.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3226,6 +3793,11 @@
           <t>Cooperativo, Per due, Dadi, Comunicazione limitata, Puzzle</t>
         </is>
       </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>In due nella cabina di un aereo: uno è il pilota, l'altro il copilota. Si piazzano i dadi sui comandi senza poter parlare, cercando di atterrare senza disastri.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3250,6 +3822,11 @@
           <t>Deckbuilder, Cooperativo, Campagna, Solitario, Fantasy</t>
         </is>
       </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>L'adattamento del videogioco: si sale una torre a piani costruendo il proprio mazzo di carte, gestendo energia e reliquie, verso boss sempre più duri. Si gioca anche da soli.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3274,6 +3851,11 @@
           <t>Gioco di carte, Controllo territorio, American, Fantasy</t>
         </is>
       </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Si mescolano due fazioni assurde — pirati zombie, dinosauri robot — e si usa il mazzo risultante per conquistare basi prima degli altri, con effetti che si combinano in modi imprevisti.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3298,6 +3880,11 @@
           <t>Eurogame, Family game, Set collection, Motore di gioco</t>
         </is>
       </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Mercanti del Rinascimento: si raccolgono gemme per comprare carte che a loro volta scontano gli acquisti successivi. Un motore che si accelera da solo, nel giro di mezz'ora.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3322,6 +3909,11 @@
           <t>Ruoli nascosti, Horror, Gioco di carte, Party game, Bluff</t>
         </is>
       </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Un'entità aliena infetta il gruppo e si diffonde passando carte di mano in mano: bisogna capire chi è ancora umano prima che il contagio prenda il sopravvento.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3346,6 +3938,11 @@
           <t>Family game, Dadi, Bambini, Classico, Scambi</t>
         </is>
       </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Si tirano due dadi con gli animali e si vedono le greggi crescere, sperando che la volpe e il lupo passino dalla parte degli altri. Si scambia per salire di specie.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3370,6 +3967,11 @@
           <t>Party game, Parole, Family game, A squadre</t>
         </is>
       </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Nomi, cose e città rivisitato: da una griglia di lettere e categorie si tirano fuori parole valide più in fretta degli altri, da soli o divisi in squadre.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3394,6 +3996,11 @@
           <t>Eurogame, Controllo territorio, Family game</t>
         </is>
       </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Versione snella di Terra Mystica: ogni popolo trasforma il terreno nel proprio e si espande, cercando di restare vicino agli altri per guadagnare di più senza rimanere senza spazio.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3418,6 +4025,11 @@
           <t>Cooperativo, Dadi, Puzzle, Solitario</t>
         </is>
       </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Un blocco di sessantaquattro dadi da smontare con metodo: la squadra li estrae, ne modifica i valori e li isola nella matrice di contenimento senza far crollare tutto.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3442,6 +4054,11 @@
           <t>Cooperativo, Gioco di carte, Solitario, Filler</t>
         </is>
       </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Quattro pile, due che salgono e due che scendono: si scartano carte quasi in silenzio, potendo scambiare pochissime informazioni, provando a svuotare il mazzo.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3466,6 +4083,11 @@
           <t>Party game, Ruoli nascosti, Bluff, Deduzione</t>
         </is>
       </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Una cellula di ribelli e qualche spia infiltrata: si vota chi mandare in missione e si osserva chi la fa fallire, discutendo e sospettando a ogni round.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3490,6 +4112,11 @@
           <t>Eurogame, Family game, Set collection, Percorsi, Classico</t>
         </is>
       </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Si collezionano carte colorate per rivendicare tratte ferroviarie e collegare le città indicate dai propri biglietti, sperando che nessuno occupi prima il passaggio chiave.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3514,6 +4141,11 @@
           <t>Family game, Quiz, Filler, Cultura generale</t>
         </is>
       </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Si inserisce una carta nella linea del tempo indovinando se l'invenzione o l'evento venga prima o dopo quelli già disposti. Vince chi si libera per primo delle sue carte.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3538,6 +4170,11 @@
           <t>Eurogame, Astratto, Family game, Piazzamento tessere</t>
         </is>
       </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Si dispongono i visitatori lungo il bordo del giardino e si sistemano le siepi scolpite in modo che, dal proprio punto di vista, la fila davanti sia la più alta e varia possibile.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3556,6 +4193,11 @@
           <t>Party game, Narrativo, Fantasy, Gioco di ruolo</t>
         </is>
       </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Un mazzo solo, due modi di usarlo: come party game fantasy fra amici oppure come piccola avventura di ruolo, con la stessa ambientazione e gli stessi personaggi.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3580,6 +4222,11 @@
           <t>Quiz, Party game, Family game, Classico, Cultura generale</t>
         </is>
       </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Il quiz per eccellenza: si gira per il tabellone rispondendo a domande di sei categorie e raccogliendo gli spicchi colorati, fino alla domanda decisiva al centro.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3604,6 +4251,11 @@
           <t>Astratto, Family game, Piazzamento tessere, Filler</t>
         </is>
       </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Si posano tessere con percorsi intrecciati e si segue la propria linea: chi finisce fuori dal tabellone o si scontra con un altro è eliminato. Vince l'ultimo rimasto in pista.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3628,6 +4280,11 @@
           <t>Deduzione, Logica, Solitario, Eurogame</t>
         </is>
       </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Una macchina logica verifica le ipotesi: si interrogano i criteri e si escludono combinazioni finché resta un solo codice possibile. Nessuna app, solo carte forate.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -3652,6 +4309,11 @@
           <t>American, Fantascienza, Controllo territorio, Negoziazione, Gioco pesante, Epico</t>
         </is>
       </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Il kolossal della fantascienza: ogni razza galattica costruisce flotte, colonizza pianeti, vota nel consiglio e tratta con le altre per arrivare per prima ai punti vittoria. Una partita occupa la giornata.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -3676,6 +4338,11 @@
           <t>Gioco di carte, Family game, Classico, Filler</t>
         </is>
       </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Si scartano carte per colore o numero, si affibbiano pescate agli avversari e si grida «Uno» quando ne resta una sola in mano — o si paga il silenzio.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -3700,6 +4367,11 @@
           <t>Gioco di carte, Family game, Filler, Solitario</t>
         </is>
       </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Uno incrociato con il gioco del golf: si dispongono sei carte coperte e si cerca di abbassare il proprio punteggio scambiandole, invece di liberarsi della mano.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -3724,6 +4396,11 @@
           <t>Gioco di carte, Party game, Umoristico, Interazione cattiva</t>
         </is>
       </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Si mette insieme una stalla di unicorni mentre gli altri provano a smantellarla con carte magiche e sabotaggi. Cattiveria pura, in versione pastello.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3748,6 +4425,11 @@
           <t>Astratto, Per due, Filler, Classico</t>
         </is>
       </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Cinque minuti di puro astratto: si accostano tessere di canale cercando di chiudere un circuito e allo stesso tempo di impedire all'avversario di farlo.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -3772,6 +4454,11 @@
           <t>Destrezza, Family game, Costruzione</t>
         </is>
       </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Si sfilano colonne di legno dai piani già costruiti e le si rimette più in alto: la torre cresce, si assottiglia e traballa, finché qualcuno la fa crollare.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -3796,6 +4483,11 @@
           <t>Party game, Destrezza, Dadi, Umoristico</t>
         </is>
       </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Stregoni che si lanciano maledizioni buffe: parlare a bassa voce, tenere un braccio alzato, non piegare i gomiti. Si accumulano punti finché si riesce a rispettarle tutte.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -3820,6 +4512,11 @@
           <t>Aste, Eurogame, Bluff</t>
         </is>
       </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Si battono all'asta reliquie leggendarie — l'Arca, la lampada di Aladino — sapendo che alcune sono falsi e che dei falsi ogni giocatore conosce solo una parte.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3844,6 +4541,11 @@
           <t>Party game, Umoristico, Per adulti</t>
         </is>
       </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Si abbina la didascalia più divertente a un'immagine e un giudice a rotazione decide quale vince. Il bello è la discussione che segue ogni verdetto.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3868,6 +4570,11 @@
           <t>Party game, Comunicazione limitata, A squadre, Deduzione</t>
         </is>
       </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Un giocatore bendato è il sognatore; gli altri gli danno indizi di una parola sola, ma alcuni mentono di proposito. Alla fine il sognatore racconta ad alta voce il sogno che ha ricostruito.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3892,6 +4599,11 @@
           <t>Movimento nascosto, Deduzione, Uno contro tutti, Storico</t>
         </is>
       </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Un giocatore è Jack lo Squartatore e si muove di nascosto annotando il percorso; gli altri sono i poliziotti che battono i vicoli di Londra per stringere il cerchio prima dell'alba.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3916,6 +4628,11 @@
           <t>Wargame, Storico, Gioco di carte, Simulazione</t>
         </is>
       </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Duelli aerei della Grande Guerra: si programmano in segreto le manovre con le carte, si rivelano simultaneamente e si spara a chi finisce nel proprio cono di tiro.</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3940,6 +4657,11 @@
           <t>Cooperativo, Miniature, American, Horror, Dadi, Solitario</t>
         </is>
       </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Cooperativo a miniature in chiave post-apocalittica: si guida una squadra di sopravvissuti in scenari infestati, si recupera equipaggiamento e si abbattono orde che crescono man mano che si diventa più forti.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3964,6 +4686,11 @@
           <t>Cooperativo, Miniature, American, Horror, Dadi, Solitario</t>
         </is>
       </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Qui gli infetti sono i supereroi Marvel: si gioca dalla parte degli zombi o contro di loro, in scenari pieni di poteri speciali e di orde che non smettono mai di arrivare.</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3988,6 +4715,11 @@
           <t>Cooperativo, Miniature, American, Horror, Dadi, Solitario</t>
         </is>
       </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Il capostipite della serie: sopravvissuti armati di quel che capita ripuliscono quartieri invasi dagli zombi. Più si sale di livello, più zombi compaiono — diventare potenti è anche il problema.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4012,6 +4744,11 @@
           <t>Dadi, Push your luck, Filler, Party game</t>
         </is>
       </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Si pescano dadi dal barattolo e si tira: cervelli da incassare, colpi di fucile che fermano tutto. Si continua finché si ha il coraggio di continuare.</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -4034,6 +4771,11 @@
       <c r="F148" t="inlineStr">
         <is>
           <t>Gioco di carte, Party game, Umoristico, Regole variabili</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Le regole cambiano di continuo perché sono esse stesse carte da giocare: obiettivi e condizioni di vittoria si trasformano mentre gli zombi si accumulano sul tavolo.</t>
         </is>
       </c>
     </row>
@@ -4357,7 +5099,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>

</xml_diff>